<commit_message>
Warehouse reference table becomes the primary engine (min/MAX ranges)
- VBA: load 'Référentiel Entrepôt' (merged box headers, min/MAX sub-row,
  X cells, '>5 & <12' text); single referenced item -> range lookup and
  combination beyond MAX; mixed orders -> capacity-fraction model with
  geometric capacities for unreferenced items; '(New)' suffix for mixed
  and unreferenced results. Referenced products no longer need dimensions.
- Python prototype mirrors the engine; tests/test_table_engine.py.
- Source workbook = user's file with the min/MAX reference sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124tbiUhdWe2XXAEg6cN3aV
</commit_message>
<xml_diff>
--- a/packaging/source/packaging_engine_mms_source.xlsx
+++ b/packaging/source/packaging_engine_mms_source.xlsx
@@ -8,11 +8,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produits" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caisses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Référentiel Entrepôt" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produits'!$A$1:$V$49</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -142,7 +143,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -165,11 +166,329 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,16 +511,98 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -783,7 +1184,7 @@
       <c r="V2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>9487</t>
         </is>
@@ -838,7 +1239,7 @@
       <c r="V3" s="12" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>9486</t>
         </is>
@@ -893,7 +1294,7 @@
       <c r="V4" s="12" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>9489</t>
         </is>
@@ -948,7 +1349,7 @@
       <c r="V5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>9488</t>
         </is>
@@ -1003,7 +1404,7 @@
       <c r="V6" s="12" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="n">
+      <c r="A7" s="22" t="n">
         <v>9492</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1056,7 +1457,7 @@
       <c r="V7" s="12" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="22" t="n">
         <v>9494</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1109,7 +1510,7 @@
       <c r="V8" s="12" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="n">
+      <c r="A9" s="22" t="n">
         <v>9495</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -1162,7 +1563,7 @@
       <c r="V9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>9263</t>
         </is>
@@ -1212,7 +1613,7 @@
       <c r="V10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>9004</t>
         </is>
@@ -1266,7 +1667,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>9509</t>
         </is>
@@ -1316,7 +1717,7 @@
       <c r="V12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n">
+      <c r="A13" s="22" t="n">
         <v>9510</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -1364,7 +1765,7 @@
       <c r="V13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>243</t>
         </is>
@@ -1754,7 +2155,7 @@
       <c r="V19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>9055</t>
         </is>
@@ -1809,7 +2210,7 @@
       <c r="V20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>9122</t>
         </is>
@@ -1859,7 +2260,7 @@
       <c r="V21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>9091</t>
         </is>
@@ -1909,7 +2310,7 @@
       <c r="V22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>9367</t>
         </is>
@@ -1959,7 +2360,7 @@
       <c r="V23" s="12" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>9366</t>
         </is>
@@ -2009,7 +2410,7 @@
       <c r="V24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>9363</t>
         </is>
@@ -2059,7 +2460,7 @@
       <c r="V25" s="12" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>9364</t>
         </is>
@@ -2109,7 +2510,7 @@
       <c r="V26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="25" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>9063</t>
         </is>
@@ -2159,7 +2560,7 @@
       <c r="V27" s="12" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>9203</t>
         </is>
@@ -2259,7 +2660,7 @@
       <c r="V29" s="12" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="25" t="n">
+      <c r="A30" s="22" t="n">
         <v>9475</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -2312,7 +2713,7 @@
       <c r="V30" s="12" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="n">
+      <c r="A31" s="22" t="n">
         <v>9476</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -2365,7 +2766,7 @@
       <c r="V31" s="12" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="n">
+      <c r="A32" s="22" t="n">
         <v>9511</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -2418,7 +2819,7 @@
       <c r="V32" s="12" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="25" t="n">
+      <c r="A33" s="22" t="n">
         <v>9512</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -2471,7 +2872,7 @@
       <c r="V33" s="12" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="25" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>9049</t>
         </is>
@@ -2526,7 +2927,7 @@
       <c r="V34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>9005</t>
         </is>
@@ -2576,7 +2977,7 @@
       <c r="V35" s="12" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="25" t="n">
+      <c r="A36" s="22" t="n">
         <v>9138</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -2810,7 +3211,7 @@
       <c r="V39" s="12" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="25" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>9120</t>
         </is>
@@ -2860,7 +3261,7 @@
       <c r="V40" s="12" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="25" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>9119</t>
         </is>
@@ -2915,7 +3316,7 @@
       <c r="V41" s="12" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>9365</t>
         </is>
@@ -3027,7 +3428,7 @@
       <c r="V43" s="12" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="25" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>9118</t>
         </is>
@@ -3077,7 +3478,7 @@
       <c r="V44" s="12" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="25" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>9130</t>
         </is>
@@ -3132,7 +3533,7 @@
       <c r="V45" s="12" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="25" t="n">
+      <c r="A46" s="22" t="n">
         <v>9491</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -3179,7 +3580,7 @@
       <c r="V46" s="12" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="25" t="n">
+      <c r="A47" s="22" t="n">
         <v>9490</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -3590,4 +3991,1163 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:T22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="52.5546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" thickBot="1"/>
+    <row r="2" ht="27.6" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Catégorie entrepôt</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="inlineStr">
+        <is>
+          <t>SKU candidats (séparés par |)</t>
+        </is>
+      </c>
+      <c r="C2" s="36" t="inlineStr">
+        <is>
+          <t>Produit (1er SKU)</t>
+        </is>
+      </c>
+      <c r="D2" s="58" t="inlineStr">
+        <is>
+          <t>Caisse Super Small</t>
+        </is>
+      </c>
+      <c r="E2" s="59" t="n"/>
+      <c r="F2" s="58" t="inlineStr">
+        <is>
+          <t>Caisse V2</t>
+        </is>
+      </c>
+      <c r="G2" s="59" t="n"/>
+      <c r="H2" s="58" t="inlineStr">
+        <is>
+          <t>Caisse V3</t>
+        </is>
+      </c>
+      <c r="I2" s="59" t="n"/>
+      <c r="J2" s="58" t="inlineStr">
+        <is>
+          <t>Caisse V4</t>
+        </is>
+      </c>
+      <c r="K2" s="59" t="n"/>
+      <c r="L2" s="58" t="inlineStr">
+        <is>
+          <t>Caisse V5</t>
+        </is>
+      </c>
+      <c r="M2" s="59" t="n"/>
+      <c r="N2" s="58" t="inlineStr">
+        <is>
+          <t>ETE Caisse V1</t>
+        </is>
+      </c>
+      <c r="O2" s="59" t="n"/>
+      <c r="P2" s="58" t="inlineStr">
+        <is>
+          <t>ETE Caisse V4</t>
+        </is>
+      </c>
+      <c r="Q2" s="59" t="n"/>
+      <c r="R2" s="58" t="inlineStr">
+        <is>
+          <t>ETE Caisse V5</t>
+        </is>
+      </c>
+      <c r="S2" s="59" t="n"/>
+      <c r="T2" s="56" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" thickBot="1">
+      <c r="A3" s="52" t="n"/>
+      <c r="B3" s="53" t="n"/>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="E3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="G3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="H3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="I3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="J3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="K3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="L3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="M3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="N3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="O3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="P3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="Q3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="R3" s="52" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="S3" s="55" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="T3" s="57" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t>40G</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>243|9138</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>Ballotin 40 g</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="47" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" s="46">
+        <f>E4+1</f>
+        <v/>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="46">
+        <f>G4+1</f>
+        <v/>
+      </c>
+      <c r="I4" s="48" t="n">
+        <v>70</v>
+      </c>
+      <c r="J4" s="46">
+        <f>I4+1</f>
+        <v/>
+      </c>
+      <c r="K4" s="47" t="n">
+        <v>80</v>
+      </c>
+      <c r="L4" s="46">
+        <f>K4+1</f>
+        <v/>
+      </c>
+      <c r="M4" s="48" t="n">
+        <v>150</v>
+      </c>
+      <c r="N4" s="49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O4" s="50" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P4" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="48" t="n">
+        <v>50</v>
+      </c>
+      <c r="R4" s="46" t="n">
+        <v>51</v>
+      </c>
+      <c r="S4" s="48" t="n">
+        <v>70</v>
+      </c>
+      <c r="T4" s="51" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>Tubes 43G</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>9055</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Tube 43 g</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" s="26">
+        <f>G5+1</f>
+        <v/>
+      </c>
+      <c r="I5" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="J5" s="26">
+        <f>I5+1</f>
+        <v/>
+      </c>
+      <c r="K5" s="27" t="n">
+        <v>60</v>
+      </c>
+      <c r="L5" s="26">
+        <f>K5+1</f>
+        <v/>
+      </c>
+      <c r="M5" s="32" t="n">
+        <v>110</v>
+      </c>
+      <c r="N5" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O5" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P5" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="R5" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="S5" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="T5" s="38" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>28G</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>9049</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>Étui Design 28 g</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" s="26">
+        <f>E6+1</f>
+        <v/>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="H6" s="26">
+        <f>G6+1</f>
+        <v/>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" s="26">
+        <f>I6+1</f>
+        <v/>
+      </c>
+      <c r="K6" s="27" t="n">
+        <v>120</v>
+      </c>
+      <c r="L6" s="26">
+        <f>K6+1</f>
+        <v/>
+      </c>
+      <c r="M6" s="32" t="n">
+        <v>200</v>
+      </c>
+      <c r="N6" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="P6" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q6" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="R6" s="26" t="n">
+        <v>61</v>
+      </c>
+      <c r="S6" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="T6" s="38" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>300G</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>9005|9263</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Écrin Chic 300 g</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="26">
+        <f>E7+1</f>
+        <v/>
+      </c>
+      <c r="G7" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="26">
+        <f>G7+1</f>
+        <v/>
+      </c>
+      <c r="I7" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="26">
+        <f>I7+1</f>
+        <v/>
+      </c>
+      <c r="K7" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="26">
+        <f>K7+1</f>
+        <v/>
+      </c>
+      <c r="M7" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="N7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="T7" s="38" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>1 KG</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>9509|9510</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Sachet vrac 1 kg</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="26">
+        <f>G8+1</f>
+        <v/>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="26">
+        <f>I8+1</f>
+        <v/>
+      </c>
+      <c r="K8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" s="26">
+        <f>K8+1</f>
+        <v/>
+      </c>
+      <c r="M8" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="T8" s="38" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>400G</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>9122|9091|9367|9366|9363|9364|9063|9365|9490|9491</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Coffret Love You 400 g</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="26">
+        <f>E9+1</f>
+        <v/>
+      </c>
+      <c r="G9" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="26">
+        <f>G9+1</f>
+        <v/>
+      </c>
+      <c r="I9" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="J9" s="26">
+        <f>I9+1</f>
+        <v/>
+      </c>
+      <c r="K9" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="L9" s="26">
+        <f>K9+1</f>
+        <v/>
+      </c>
+      <c r="M9" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="N9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="R9" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="S9" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="T9" s="38" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>BULK 1.5</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>9004|9120|9119|9118</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Sachet vrac 1,5 kg</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="26">
+        <f>G10+1</f>
+        <v/>
+      </c>
+      <c r="I10" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="26">
+        <f>I10+1</f>
+        <v/>
+      </c>
+      <c r="K10" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" s="26">
+        <f>K10+1</f>
+        <v/>
+      </c>
+      <c r="M10" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="T10" s="38" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Distributeur Fun Machine</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>9130</v>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Distributeur Fun Machine</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="26">
+        <f>I11+1</f>
+        <v/>
+      </c>
+      <c r="K11" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" s="26">
+        <f>K11+1</f>
+        <v/>
+      </c>
+      <c r="M11" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O11" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="R11" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S11" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T11" s="38" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>500G</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>9203</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Boîte Cœur 500 g</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="26">
+        <f>E12+1</f>
+        <v/>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="26">
+        <f>G12+1</f>
+        <v/>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="26">
+        <f>I12+1</f>
+        <v/>
+      </c>
+      <c r="K12" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" s="26">
+        <f>K12+1</f>
+        <v/>
+      </c>
+      <c r="M12" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="N12" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="R12" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="S12" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="T12" s="38" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>ROUNDCOPACK</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>9488|9487|9486|9489|9492|9494|9495</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Boîte ronde</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="26">
+        <f>E13+1</f>
+        <v/>
+      </c>
+      <c r="G13" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H13" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I13" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="K13" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="L13" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N13" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q13" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="R13" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S13" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" s="38" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Distributer 3 en 1</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>9475|9476|9511|9512</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Distributer 3 en 1</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J14" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="26">
+        <f>K14+1</f>
+        <v/>
+      </c>
+      <c r="M14" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O14" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Q14" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="S14" s="33" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" s="38" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="n"/>
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="D15" s="26" t="n"/>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="26" t="n"/>
+      <c r="I15" s="27" t="n"/>
+      <c r="J15" s="26" t="n"/>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="26" t="n"/>
+      <c r="M15" s="27" t="n"/>
+      <c r="N15" s="26" t="n"/>
+      <c r="O15" s="27" t="n"/>
+      <c r="P15" s="26" t="n"/>
+      <c r="Q15" s="27" t="n"/>
+      <c r="R15" s="26" t="n"/>
+      <c r="S15" s="27" t="n"/>
+      <c r="T15" s="38" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="n"/>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="23" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="26" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="26" t="n"/>
+      <c r="M16" s="27" t="n"/>
+      <c r="N16" s="26" t="n"/>
+      <c r="O16" s="27" t="n"/>
+      <c r="P16" s="26" t="n"/>
+      <c r="Q16" s="27" t="n"/>
+      <c r="R16" s="26" t="n"/>
+      <c r="S16" s="27" t="n"/>
+      <c r="T16" s="38" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="n"/>
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="26" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="26" t="n"/>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="26" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="26" t="n"/>
+      <c r="M17" s="27" t="n"/>
+      <c r="N17" s="26" t="n"/>
+      <c r="O17" s="27" t="n"/>
+      <c r="P17" s="26" t="n"/>
+      <c r="Q17" s="27" t="n"/>
+      <c r="R17" s="26" t="n"/>
+      <c r="S17" s="27" t="n"/>
+      <c r="T17" s="38" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="37" t="n"/>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="23" t="n"/>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="26" t="n"/>
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="26" t="n"/>
+      <c r="K18" s="27" t="n"/>
+      <c r="L18" s="26" t="n"/>
+      <c r="M18" s="27" t="n"/>
+      <c r="N18" s="26" t="n"/>
+      <c r="O18" s="27" t="n"/>
+      <c r="P18" s="26" t="n"/>
+      <c r="Q18" s="27" t="n"/>
+      <c r="R18" s="26" t="n"/>
+      <c r="S18" s="27" t="n"/>
+      <c r="T18" s="38" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="n"/>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="26" t="n"/>
+      <c r="I19" s="27" t="n"/>
+      <c r="J19" s="26" t="n"/>
+      <c r="K19" s="27" t="n"/>
+      <c r="L19" s="26" t="n"/>
+      <c r="M19" s="27" t="n"/>
+      <c r="N19" s="26" t="n"/>
+      <c r="O19" s="27" t="n"/>
+      <c r="P19" s="26" t="n"/>
+      <c r="Q19" s="27" t="n"/>
+      <c r="R19" s="26" t="n"/>
+      <c r="S19" s="27" t="n"/>
+      <c r="T19" s="38" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1" thickBot="1">
+      <c r="A20" s="39" t="n"/>
+      <c r="B20" s="40" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="30" t="n"/>
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="30" t="n"/>
+      <c r="I20" s="31" t="n"/>
+      <c r="J20" s="30" t="n"/>
+      <c r="K20" s="31" t="n"/>
+      <c r="L20" s="30" t="n"/>
+      <c r="M20" s="31" t="n"/>
+      <c r="N20" s="30" t="n"/>
+      <c r="O20" s="31" t="n"/>
+      <c r="P20" s="30" t="n"/>
+      <c r="Q20" s="31" t="n"/>
+      <c r="R20" s="30" t="n"/>
+      <c r="S20" s="31" t="n"/>
+      <c r="T20" s="42" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Lecture : nombre MAX d'articles de la catégorie que la caisse peut contenir (« jusqu'à »). X (gris) = caisse non autorisée pour cet article.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Cellules jaunes modifiables : SKU candidats (le 1er sert au calcul) et quantités. Comparaison : python3 tools/compare_entrepot.py &lt;classeur&gt; (lit cette feuille).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="P2:Q2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>